<commit_message>
Improve algorithm and achieve 100% test coverage
</commit_message>
<xml_diff>
--- a/PSP.xlsx
+++ b/PSP.xlsx
@@ -422,10 +422,10 @@
   <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -464,7 +464,9 @@
       <c r="C2" t="n">
         <v>30</v>
       </c>
-      <c r="D2" t="inlineStr"/>
+      <c r="D2" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -480,7 +482,9 @@
       <c r="C3" t="n">
         <v>20</v>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -496,7 +500,9 @@
       <c r="C4" t="n">
         <v>120</v>
       </c>
-      <c r="D4" t="inlineStr"/>
+      <c r="D4" t="n">
+        <v>150</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -512,7 +518,9 @@
       <c r="C5" t="n">
         <v>60</v>
       </c>
-      <c r="D5" t="inlineStr"/>
+      <c r="D5" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -528,7 +536,9 @@
       <c r="C6" t="n">
         <v>30</v>
       </c>
-      <c r="D6" t="inlineStr"/>
+      <c r="D6" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -544,7 +554,9 @@
       <c r="C7" t="n">
         <v>30</v>
       </c>
-      <c r="D7" t="inlineStr"/>
+      <c r="D7" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -560,7 +572,9 @@
       <c r="C8" t="n">
         <v>60</v>
       </c>
-      <c r="D8" t="inlineStr"/>
+      <c r="D8" t="n">
+        <v>70</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -576,7 +590,9 @@
       <c r="C9" t="n">
         <v>300</v>
       </c>
-      <c r="D9" t="inlineStr"/>
+      <c r="D9" t="n">
+        <v>360</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -592,7 +608,9 @@
       <c r="C10" t="n">
         <v>60</v>
       </c>
-      <c r="D10" t="inlineStr"/>
+      <c r="D10" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -608,7 +626,9 @@
       <c r="C11" t="n">
         <v>180</v>
       </c>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="n">
+        <v>200</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -624,7 +644,9 @@
       <c r="C12" t="n">
         <v>60</v>
       </c>
-      <c r="D12" t="inlineStr"/>
+      <c r="D12" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -640,7 +662,9 @@
       <c r="C13" t="n">
         <v>20</v>
       </c>
-      <c r="D13" t="inlineStr"/>
+      <c r="D13" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -656,7 +680,9 @@
       <c r="C14" t="n">
         <v>30</v>
       </c>
-      <c r="D14" t="inlineStr"/>
+      <c r="D14" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -664,12 +690,13 @@
           <t>合计</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15">
         <f>SUM(C2:C14)</f>
         <v/>
       </c>
-      <c r="D15" t="inlineStr"/>
+      <c r="D15" t="n">
+        <v>1110</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>